<commit_message>
Catttle modeled results created
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-04-29-cattle-slurry-retrail/2026-04-29-CattleSlurryRetry-slurry.xlsx
+++ b/Lab-trails/2026-04-29-cattle-slurry-retrail/2026-04-29-CattleSlurryRetry-slurry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-04-29-cattle-slurry-retrail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DFB7B9-65B1-4CF6-8F29-44A0684698F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F347594F-078D-4625-B8F4-A321F5E03EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAN" sheetId="1" r:id="rId1"/>
@@ -1109,7 +1109,8 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="5" width="13.33203125" customWidth="1"/>
+    <col min="2" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">

</xml_diff>